<commit_message>
fix: correction erreurs SUSHI et préparation release 1.2.0-snapshot-2
- Correction du slicing qualification[attributionParticuliere] : binding déplacé de code vers code.coding pour correspondre au discriminateur FRCore
- Correction du conflit meta.profile[fr-canonical] : remplacement de Canonical(fr-core-xxx) par les URLs versionnées |2.2.0 dans les 16 exemples DP/DR
- Version bump 1.2.0-snapshot-1 → 1.2.0-snapshot-2
- Mise à jour du changelog (changes.md) avec les PRs #304, #306, #307

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> b48b5d6c7ef30b35f4df3071237aca0b597bbd4e
</commit_message>
<xml_diff>
--- a/nr-update-frcore-2.2.0/ig/CodeSystem-as-cs-organization-types.xlsx
+++ b/nr-update-frcore-2.2.0/ig/CodeSystem-as-cs-organization-types.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.2.0-snapshot-1</t>
+    <t>1.2.0-snapshot-2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-18T11:49:33+00:00</t>
+    <t>2026-06-18T12:07:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>